<commit_message>
Bug!!! fix promt roadmap + excel
</commit_message>
<xml_diff>
--- a/DemoImportCourses.xlsx
+++ b/DemoImportCourses.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>STT</t>
   </si>
@@ -35,64 +35,61 @@
     <t>Chuẩn đầu ra</t>
   </si>
   <si>
-    <t>PRN211</t>
-  </si>
-  <si>
-    <t>Basic Cross-Platform Application Programming</t>
-  </si>
-  <si>
-    <t>C#, .NET, Entity Framework, LINQ</t>
-  </si>
-  <si>
-    <t>Hiểu ngôn ngữ C# cơ bản; Lập trình hướng đối tượng với .NET; Truy vấn DB bằng Entity Framework Core; Sử dụng LINQ nâng cao</t>
-  </si>
-  <si>
-    <t>PRN221</t>
-  </si>
-  <si>
-    <t>Advanced Cross-Platform Application Programming</t>
-  </si>
-  <si>
-    <t>C#, .NET, WPF, SignalR</t>
-  </si>
-  <si>
-    <t>Lập trình desktop với WPF; Xây dựng ứng dụng thời gian thực bằng SignalR</t>
-  </si>
-  <si>
-    <t>PRN231</t>
-  </si>
-  <si>
-    <t>Web Application Development</t>
-  </si>
-  <si>
-    <t>ASP.NET Core, RESTful API, Web API</t>
-  </si>
-  <si>
-    <t>Xây dựng web app với ASP.NET Core; Thiết kế RESTful Web API chuẩn chỉnh</t>
-  </si>
-  <si>
-    <t>SWE102</t>
-  </si>
-  <si>
-    <t>Introduction to Software Engineering</t>
-  </si>
-  <si>
-    <t>Software Process, Git, Requirements Engineering</t>
-  </si>
-  <si>
-    <t>Nắm rõ các quy trình sản xuất phần mềm; Sử dụng Git quản lý mã nguồn; Phân tích và viết đặc tả yêu cầu phần mềm</t>
-  </si>
-  <si>
-    <t>SWD392</t>
-  </si>
-  <si>
-    <t>Software Architecture and Design</t>
-  </si>
-  <si>
-    <t>UML, Design Patterns, Software Architecture</t>
-  </si>
-  <si>
-    <t>Vẽ và thiết kế hệ thống bằng UML; Áp dụng các Design Patterns thông dụng; Phân tích cấu trúc kiến trúc phần mềm</t>
+    <t>Môn học nền tảng</t>
+  </si>
+  <si>
+    <t>PRJ301</t>
+  </si>
+  <si>
+    <t>Java Web Application Development</t>
+  </si>
+  <si>
+    <t>Servlet, JSP, MVC Architecture</t>
+  </si>
+  <si>
+    <t>Hiểu kiến trúc MVC; Phát triển ứng dụng Web động bằng JSP và Servlet; Triển khai ứng dụng Web Java</t>
+  </si>
+  <si>
+    <t>False</t>
+  </si>
+  <si>
+    <t>FER202</t>
+  </si>
+  <si>
+    <t>Front-End Web Development with React</t>
+  </si>
+  <si>
+    <t>React.js, Responsive Web Design, JavaScript</t>
+  </si>
+  <si>
+    <t>Xây dựng giao diện web SPA bằng ReactJS; Quản lý state; Sử dụng React Hooks</t>
+  </si>
+  <si>
+    <t>PRM393</t>
+  </si>
+  <si>
+    <t>Mobile Application Development</t>
+  </si>
+  <si>
+    <t>Flutter, Dart Programming, Android Development</t>
+  </si>
+  <si>
+    <t>Lập trình ứng dụng di động đa nền tảng bằng Flutter &amp; Dart; Thiết kế giao diện di động</t>
+  </si>
+  <si>
+    <t>CSD201</t>
+  </si>
+  <si>
+    <t>Data Structures and Algorithms</t>
+  </si>
+  <si>
+    <t>Data Structures, Algorithm Design &amp; Analysis, OOP</t>
+  </si>
+  <si>
+    <t>Cài đặt các cấu trúc dữ liệu cơ bản như Tree, Graph, Stack, Queue; Đánh giá độ phức tạp thuật toán</t>
+  </si>
+  <si>
+    <t>True</t>
   </si>
 </sst>
 </file>
@@ -166,7 +163,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1" style="3"/>
@@ -176,6 +173,7 @@
     <col min="5" max="5" width="18" customWidth="1" style="3"/>
     <col min="6" max="6" width="45" customWidth="1"/>
     <col min="7" max="7" width="60" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -200,16 +198,19 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="4">
         <v>3</v>
@@ -218,10 +219,13 @@
         <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -229,10 +233,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="4">
         <v>3</v>
@@ -241,10 +245,13 @@
         <v>90</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -252,10 +259,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="4">
         <v>3</v>
@@ -264,10 +271,13 @@
         <v>90</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -275,45 +285,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D5" s="4">
         <v>3</v>
       </c>
       <c r="E5" s="4">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="4">
-        <v>3</v>
-      </c>
-      <c r="E6" s="4">
-        <v>60</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>